<commit_message>
penambahan point upgrade os
</commit_message>
<xml_diff>
--- a/assets/excel/Data Kendala SE.xlsx
+++ b/assets/excel/Data Kendala SE.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="194">
   <si>
     <t>NO</t>
   </si>
@@ -83,7 +83,7 @@
     <t>RAYA CISOKA KM 1</t>
   </si>
   <si>
-    <t>Tidak dapat aktivasi sudah memkasi lisensi yang tertera, keterangan already use on another device</t>
+    <t>Tidak dapat aktivasi sudah memakai lisensi yang tertera, keterangan already use on another device</t>
   </si>
   <si>
     <t>2024-09-27</t>
@@ -122,6 +122,114 @@
     <t>2024-10-08</t>
   </si>
   <si>
+    <t>TUB4</t>
+  </si>
+  <si>
+    <t>PABUARAN TIGARAKSA</t>
+  </si>
+  <si>
+    <t>EDC MANDIRI MERK INGENICO TIDAK SUPPORT ONLINE</t>
+  </si>
+  <si>
+    <t>2024-10-10</t>
+  </si>
+  <si>
+    <t>TCR5</t>
+  </si>
+  <si>
+    <t>CISOKA CARINGIN</t>
+  </si>
+  <si>
+    <t>SUDAH DI AKTIVASI ULANG DAN BERHASIL, TETAPI MASIH MUNCUL DI WEB</t>
+  </si>
+  <si>
+    <t>2024-10-11</t>
+  </si>
+  <si>
+    <t>TS3E</t>
+  </si>
+  <si>
+    <t>HYBRID TALAGA BESTARI</t>
+  </si>
+  <si>
+    <t>SUDAH DI AKTIVASI ULANG DAN BERHASIL, UNTUK CPU PERNAH DI TUKAR OLEH AS KE GA. ( MASIH MUCUL DI WEB )</t>
+  </si>
+  <si>
+    <t>FD5K</t>
+  </si>
+  <si>
+    <t>BUGEL TIGARAKSA</t>
+  </si>
+  <si>
+    <t>Sudah aktivasi tetpi masih muncul DI WEB</t>
+  </si>
+  <si>
+    <t>2024-10-17</t>
+  </si>
+  <si>
+    <t>F5CF</t>
+  </si>
+  <si>
+    <t>REST AREA KM 45</t>
+  </si>
+  <si>
+    <t>EDC BCA RUSAK TIDAK DAPAT HIDUP HARUS GANTI EDC</t>
+  </si>
+  <si>
+    <t>2024-10-16</t>
+  </si>
+  <si>
+    <t>edc bca offline</t>
+  </si>
+  <si>
+    <t>EDC MANDIRI TIDAK SUPPORT ONLINE</t>
+  </si>
+  <si>
+    <t>TP1Q</t>
+  </si>
+  <si>
+    <t>CISOKA MEGU</t>
+  </si>
+  <si>
+    <t>EDC BCA RUSAK SUDAH KONFIRMASI KE TEAM VIRTUAL</t>
+  </si>
+  <si>
+    <t>TYWO</t>
+  </si>
+  <si>
+    <t>CISOKA TIGARAKSA</t>
+  </si>
+  <si>
+    <t>SUDAH DI INSTALL ULANG SESUAI LISENSI DI CPU</t>
+  </si>
+  <si>
+    <t>TAK1</t>
+  </si>
+  <si>
+    <t>RAYA SODONG</t>
+  </si>
+  <si>
+    <t>EDC BCA KETERANGAN NO SIM CARD</t>
+  </si>
+  <si>
+    <t>2024-10-19</t>
+  </si>
+  <si>
+    <t>FHXE</t>
+  </si>
+  <si>
+    <t>RSUD BALARAJA</t>
+  </si>
+  <si>
+    <t>WINDOWS SUDAH DI AKTIVASI TETAPI MASIH TERDAFTAR SEBAGAI TOKO BELUM AKTIVASI DI WEB</t>
+  </si>
+  <si>
+    <t>2024-10-26</t>
+  </si>
+  <si>
+    <t>EDC BCA TIDAK ONLINE , HANK TIDAK MAU HIDUP KETERANGAN KEY INJECTION</t>
+  </si>
+  <si>
     <t>AHMAD SOFYAN</t>
   </si>
   <si>
@@ -203,6 +311,18 @@
     <t>tidak ada licensy ( KOMPUTER CADANGAN GA )</t>
   </si>
   <si>
+    <t>TJIQ</t>
+  </si>
+  <si>
+    <t>TMP TARUNA</t>
+  </si>
+  <si>
+    <t>KOMPUTER STATION 09 SUDAH DI LEPAS</t>
+  </si>
+  <si>
+    <t>2024-10-24</t>
+  </si>
+  <si>
     <t>DEDE HERMANSYAH</t>
   </si>
   <si>
@@ -248,22 +368,19 @@
     <t>2024-10-04</t>
   </si>
   <si>
-    <t>edc bca offline</t>
-  </si>
-  <si>
     <t>ILHAM M FIRDAUS</t>
   </si>
   <si>
-    <t>FK01</t>
-  </si>
-  <si>
-    <t>BENTENG BETAWI II</t>
-  </si>
-  <si>
-    <t>PORT MESIN EDC MANDIRI DUGAAN RUSAK/SUDAH KENDOR, SUDAH INFO KE VIRTUAL</t>
-  </si>
-  <si>
-    <t>2024-09-23</t>
+    <t>FVKQ</t>
+  </si>
+  <si>
+    <t>SPRINGWOOD</t>
+  </si>
+  <si>
+    <t>EDC BCA TIDAK BISA MEMBACA CHIP KARTU DEBIT</t>
+  </si>
+  <si>
+    <t>2024-10-09</t>
   </si>
   <si>
     <t>TKG8</t>
@@ -272,10 +389,22 @@
     <t>KELAPA INDAH</t>
   </si>
   <si>
-    <t>MESIN EDC BCA MATI TIDAK BISA NYALA</t>
-  </si>
-  <si>
-    <t>2024-10-07</t>
+    <t>EDC BCA TIDAK ADA SINYAL DAN TIDAK BISA SETTLEMENT</t>
+  </si>
+  <si>
+    <t>2024-10-14</t>
+  </si>
+  <si>
+    <t>T0DA</t>
+  </si>
+  <si>
+    <t>RUKO AZORES BLOK B17A NO.16&amp;17</t>
+  </si>
+  <si>
+    <t>PORT USB DI MESIN EDC MANDIRI SUDAH GOYANG / PATAH, MENYEBABKAN TIDAK ONLINE</t>
+  </si>
+  <si>
+    <t>2024-10-29</t>
   </si>
   <si>
     <t>JAMHARA PARPANI</t>
@@ -419,33 +548,15 @@
     <t>tidak bisa aktivasi windows ulang, pilihan change product key tidah muncul indikasi os error</t>
   </si>
   <si>
-    <t>F9GD</t>
-  </si>
-  <si>
-    <t>MUNJUL SOLEAR</t>
-  </si>
-  <si>
-    <t>sudah aktivasi sesuai license pengerjaan upgrade os dari 7 ke 10 agar sesuai license win 10</t>
-  </si>
-  <si>
-    <t>T17I</t>
-  </si>
-  <si>
-    <t>SUDIRMAN INDAH</t>
+    <t>TAUT</t>
+  </si>
+  <si>
+    <t>KORELET</t>
   </si>
   <si>
     <t>edc bca seting offline kabel ecr biru error, butuh kabel ecr baru castles</t>
   </si>
   <si>
-    <t>2024-10-09</t>
-  </si>
-  <si>
-    <t>TAUT</t>
-  </si>
-  <si>
-    <t>KORELET</t>
-  </si>
-  <si>
     <t>PRADITYA RIYAN VIVALDI</t>
   </si>
   <si>
@@ -471,6 +582,21 @@
   </si>
   <si>
     <t>2024-08-25</t>
+  </si>
+  <si>
+    <t>RAMADHAN SAPUTRA</t>
+  </si>
+  <si>
+    <t>T34E</t>
+  </si>
+  <si>
+    <t>SANGEGO BAYUR</t>
+  </si>
+  <si>
+    <t>Status komputer cadangan GA, tidak di temukan lisensi pada komputer</t>
+  </si>
+  <si>
+    <t>2024-10-13</t>
   </si>
 </sst>
 </file>
@@ -809,7 +935,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1017,42 +1143,42 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="B8">
-        <v>2012056661</v>
+        <v>2012110141</v>
       </c>
       <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s">
         <v>35</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>36</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>37</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8" t="s">
         <v>38</v>
       </c>
-      <c r="G8">
-        <v>4</v>
-      </c>
-      <c r="H8" t="s">
-        <v>28</v>
-      </c>
       <c r="I8" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="B9">
-        <v>2012056661</v>
+        <v>2012110141</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="D9" t="s">
         <v>39</v>
@@ -1061,114 +1187,114 @@
         <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>38</v>
-      </c>
-      <c r="G9" t="s">
-        <v>18</v>
+        <v>41</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="I9" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10">
-        <v>55</v>
+        <v>120</v>
       </c>
       <c r="B10">
-        <v>2012056661</v>
+        <v>2012110141</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10">
+        <v>6</v>
+      </c>
+      <c r="H10" t="s">
         <v>42</v>
       </c>
-      <c r="F10" t="s">
-        <v>38</v>
-      </c>
-      <c r="G10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" t="s">
-        <v>28</v>
-      </c>
       <c r="I10" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11">
-        <v>56</v>
+        <v>124</v>
       </c>
       <c r="B11">
-        <v>2012056661</v>
+        <v>2012110141</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E11" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F11" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" t="s">
-        <v>18</v>
+        <v>48</v>
+      </c>
+      <c r="G11">
+        <v>2</v>
       </c>
       <c r="H11" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12">
-        <v>69</v>
+        <v>125</v>
       </c>
       <c r="B12">
-        <v>2015111644</v>
+        <v>2012110141</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F12" t="s">
-        <v>48</v>
-      </c>
-      <c r="G12" t="s">
-        <v>18</v>
+        <v>52</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
       </c>
       <c r="H12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I12" t="s">
-        <v>19</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13">
-        <v>79</v>
+        <v>126</v>
       </c>
       <c r="B13">
-        <v>2015111644</v>
+        <v>2012110141</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="D13" t="s">
         <v>50</v>
@@ -1177,56 +1303,56 @@
         <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H13" t="s">
         <v>53</v>
       </c>
       <c r="I13" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="B14">
-        <v>2015111644</v>
+        <v>2012110141</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14" t="s">
+        <v>49</v>
+      </c>
+      <c r="I14" t="s">
         <v>54</v>
-      </c>
-      <c r="E14" t="s">
-        <v>55</v>
-      </c>
-      <c r="F14" t="s">
-        <v>56</v>
-      </c>
-      <c r="G14" t="s">
-        <v>18</v>
-      </c>
-      <c r="H14" t="s">
-        <v>57</v>
-      </c>
-      <c r="I14" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15">
-        <v>87</v>
+        <v>128</v>
       </c>
       <c r="B15">
-        <v>2013026705</v>
+        <v>2012110141</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="D15" t="s">
         <v>59</v>
@@ -1237,11 +1363,11 @@
       <c r="F15" t="s">
         <v>61</v>
       </c>
-      <c r="G15" t="s">
-        <v>18</v>
+      <c r="G15">
+        <v>2</v>
       </c>
       <c r="H15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="I15" t="s">
         <v>14</v>
@@ -1249,57 +1375,57 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16">
-        <v>43</v>
+        <v>129</v>
       </c>
       <c r="B16">
-        <v>2013008437</v>
+        <v>2012110141</v>
       </c>
       <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s">
         <v>62</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>63</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>64</v>
-      </c>
-      <c r="F16" t="s">
-        <v>65</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
       <c r="H16" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="I16" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17">
-        <v>44</v>
+        <v>131</v>
       </c>
       <c r="B17">
-        <v>2013008437</v>
+        <v>2012110141</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>9</v>
       </c>
       <c r="D17" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E17" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F17" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17" t="s">
-        <v>23</v>
+        <v>69</v>
       </c>
       <c r="I17" t="s">
         <v>24</v>
@@ -1307,318 +1433,318 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18">
-        <v>58</v>
+        <v>132</v>
       </c>
       <c r="B18">
-        <v>2013008437</v>
+        <v>2012110141</v>
       </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>9</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="F18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G18">
         <v>1</v>
       </c>
       <c r="H18" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="I18" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B19">
-        <v>2013008437</v>
+        <v>2012056661</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D19" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E19" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F19" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H19" t="s">
         <v>28</v>
       </c>
       <c r="I19" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="B20">
-        <v>2013008437</v>
+        <v>2012056661</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D20" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="E20" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F20" t="s">
-        <v>71</v>
-      </c>
-      <c r="G20">
-        <v>9</v>
+        <v>74</v>
+      </c>
+      <c r="G20" t="s">
+        <v>18</v>
       </c>
       <c r="H20" t="s">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="I20" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="B21">
-        <v>2013008437</v>
+        <v>2012056661</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E21" t="s">
+        <v>78</v>
+      </c>
+      <c r="F21" t="s">
         <v>74</v>
       </c>
-      <c r="F21" t="s">
-        <v>75</v>
-      </c>
-      <c r="G21">
-        <v>3</v>
+      <c r="G21" t="s">
+        <v>18</v>
       </c>
       <c r="H21" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="I21" t="s">
-        <v>77</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22">
-        <v>91</v>
+        <v>56</v>
       </c>
       <c r="B22">
-        <v>2013008437</v>
+        <v>2012056661</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E22" t="s">
+        <v>80</v>
+      </c>
+      <c r="F22" t="s">
         <v>74</v>
       </c>
-      <c r="F22" t="s">
-        <v>75</v>
-      </c>
-      <c r="G22">
-        <v>5</v>
+      <c r="G22" t="s">
+        <v>18</v>
       </c>
       <c r="H22" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="I22" t="s">
-        <v>77</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="B23">
-        <v>2015076044</v>
+        <v>2015111644</v>
       </c>
       <c r="C23" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D23" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E23" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F23" t="s">
-        <v>81</v>
-      </c>
-      <c r="G23">
-        <v>1</v>
+        <v>84</v>
+      </c>
+      <c r="G23" t="s">
+        <v>18</v>
       </c>
       <c r="H23" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I23" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="B24">
-        <v>2015076044</v>
+        <v>2015111644</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E24" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F24" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H24" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I24" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25">
-        <v>36</v>
+        <v>81</v>
       </c>
       <c r="B25">
-        <v>2013037005</v>
+        <v>2015111644</v>
       </c>
       <c r="C25" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D25" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E25" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F25" t="s">
-        <v>90</v>
-      </c>
-      <c r="G25">
-        <v>1</v>
+        <v>92</v>
+      </c>
+      <c r="G25" t="s">
+        <v>18</v>
       </c>
       <c r="H25" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I25" t="s">
-        <v>77</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26">
-        <v>50</v>
+        <v>87</v>
       </c>
       <c r="B26">
-        <v>2013037005</v>
+        <v>2013026705</v>
       </c>
       <c r="C26" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D26" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E26" t="s">
+        <v>96</v>
+      </c>
+      <c r="F26" t="s">
+        <v>97</v>
+      </c>
+      <c r="G26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H26" t="s">
         <v>93</v>
       </c>
-      <c r="F26" t="s">
-        <v>94</v>
-      </c>
-      <c r="G26">
-        <v>1</v>
-      </c>
-      <c r="H26" t="s">
-        <v>95</v>
-      </c>
       <c r="I26" t="s">
-        <v>96</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27">
-        <v>51</v>
+        <v>130</v>
       </c>
       <c r="B27">
-        <v>2013037005</v>
+        <v>2013026705</v>
       </c>
       <c r="C27" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G27">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H27" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I27" t="s">
-        <v>96</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B28">
-        <v>2013037005</v>
+        <v>2013008437</v>
       </c>
       <c r="C28" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D28" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E28" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F28" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G28">
         <v>1</v>
       </c>
       <c r="H28" t="s">
-        <v>95</v>
+        <v>23</v>
       </c>
       <c r="I28" t="s">
         <v>24</v>
@@ -1626,13 +1752,13 @@
     </row>
     <row r="29" spans="1:9">
       <c r="A29">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="B29">
-        <v>2013037005</v>
+        <v>2013008437</v>
       </c>
       <c r="C29" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D29" t="s">
         <v>103</v>
@@ -1644,329 +1770,329 @@
         <v>105</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I29" t="s">
-        <v>106</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B30">
-        <v>2013037005</v>
+        <v>2013008437</v>
       </c>
       <c r="C30" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D30" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="E30" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="F30" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="G30">
         <v>2</v>
       </c>
       <c r="H30" t="s">
-        <v>107</v>
+        <v>28</v>
       </c>
       <c r="I30" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="B31">
-        <v>2013037005</v>
+        <v>2013008437</v>
       </c>
       <c r="C31" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D31" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E31" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F31" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H31" t="s">
-        <v>28</v>
+        <v>112</v>
       </c>
       <c r="I31" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="B32">
-        <v>2013037005</v>
+        <v>2013008437</v>
       </c>
       <c r="C32" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D32" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E32" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F32" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H32" t="s">
-        <v>49</v>
+        <v>116</v>
       </c>
       <c r="I32" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="1:9">
       <c r="A33">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="B33">
-        <v>2013037005</v>
+        <v>2013008437</v>
       </c>
       <c r="C33" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D33" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E33" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F33" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G33">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H33" t="s">
-        <v>49</v>
+        <v>116</v>
       </c>
       <c r="I33" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34" spans="1:9">
       <c r="A34">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="B34">
-        <v>2013037005</v>
+        <v>2015076044</v>
       </c>
       <c r="C34" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="D34" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="E34" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="F34" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="G34">
         <v>1</v>
       </c>
       <c r="H34" t="s">
-        <v>95</v>
+        <v>121</v>
       </c>
       <c r="I34" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:9">
       <c r="A35">
-        <v>85</v>
+        <v>123</v>
       </c>
       <c r="B35">
-        <v>2013037005</v>
+        <v>2015076044</v>
       </c>
       <c r="C35" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="D35" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="E35" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="F35" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="G35">
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>57</v>
+        <v>125</v>
       </c>
       <c r="I35" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:9">
       <c r="A36">
-        <v>86</v>
+        <v>133</v>
       </c>
       <c r="B36">
-        <v>2013037005</v>
+        <v>2015076044</v>
       </c>
       <c r="C36" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="D36" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E36" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="F36" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="G36">
         <v>1</v>
       </c>
       <c r="H36" t="s">
-        <v>57</v>
+        <v>129</v>
       </c>
       <c r="I36" t="s">
-        <v>77</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:9">
       <c r="A37">
-        <v>92</v>
+        <v>36</v>
       </c>
       <c r="B37">
         <v>2013037005</v>
       </c>
       <c r="C37" t="s">
-        <v>87</v>
+        <v>130</v>
       </c>
       <c r="D37" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="E37" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="F37" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="G37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H37" t="s">
-        <v>76</v>
+        <v>134</v>
       </c>
       <c r="I37" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="38" spans="1:9">
       <c r="A38">
-        <v>93</v>
+        <v>50</v>
       </c>
       <c r="B38">
         <v>2013037005</v>
       </c>
       <c r="C38" t="s">
-        <v>87</v>
+        <v>130</v>
       </c>
       <c r="D38" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="E38" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="F38" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="G38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H38" t="s">
-        <v>57</v>
+        <v>138</v>
       </c>
       <c r="I38" t="s">
-        <v>24</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:9">
       <c r="A39">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="B39">
         <v>2013037005</v>
       </c>
       <c r="C39" t="s">
-        <v>87</v>
+        <v>130</v>
       </c>
       <c r="D39" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="E39" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="F39" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="G39">
         <v>2</v>
       </c>
       <c r="H39" t="s">
-        <v>57</v>
+        <v>138</v>
       </c>
       <c r="I39" t="s">
-        <v>24</v>
+        <v>139</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40">
-        <v>95</v>
+        <v>52</v>
       </c>
       <c r="B40">
         <v>2013037005</v>
       </c>
       <c r="C40" t="s">
-        <v>87</v>
+        <v>130</v>
       </c>
       <c r="D40" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="E40" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="F40" t="s">
-        <v>123</v>
-      </c>
-      <c r="G40" t="s">
-        <v>18</v>
+        <v>145</v>
+      </c>
+      <c r="G40">
+        <v>1</v>
       </c>
       <c r="H40" t="s">
-        <v>57</v>
+        <v>138</v>
       </c>
       <c r="I40" t="s">
         <v>24</v>
@@ -1974,39 +2100,39 @@
     </row>
     <row r="41" spans="1:9">
       <c r="A41">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="B41">
         <v>2013037005</v>
       </c>
       <c r="C41" t="s">
-        <v>87</v>
+        <v>130</v>
       </c>
       <c r="D41" t="s">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="E41" t="s">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="F41" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
       <c r="G41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>129</v>
+        <v>28</v>
       </c>
       <c r="I41" t="s">
-        <v>24</v>
+        <v>149</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="B42">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C42" t="s">
         <v>130</v>
@@ -2021,39 +2147,39 @@
         <v>133</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H42" t="s">
-        <v>49</v>
+        <v>150</v>
       </c>
       <c r="I42" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="B43">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C43" t="s">
         <v>130</v>
       </c>
       <c r="D43" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="E43" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="F43" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="G43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H43" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="I43" t="s">
         <v>14</v>
@@ -2061,582 +2187,437 @@
     </row>
     <row r="44" spans="1:9">
       <c r="A44">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="B44">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C44" t="s">
         <v>130</v>
       </c>
       <c r="D44" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="E44" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="F44" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="G44">
         <v>1</v>
       </c>
       <c r="H44" t="s">
-        <v>140</v>
+        <v>85</v>
       </c>
       <c r="I44" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="B45">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C45" t="s">
         <v>130</v>
       </c>
       <c r="D45" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="E45" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="F45" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="G45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H45" t="s">
-        <v>140</v>
+        <v>85</v>
       </c>
       <c r="I45" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="B46">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C46" t="s">
         <v>130</v>
       </c>
       <c r="D46" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="E46" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="F46" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="G46">
         <v>1</v>
       </c>
       <c r="H46" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I46" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="B47">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C47" t="s">
         <v>130</v>
       </c>
       <c r="D47" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="E47" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="F47" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="G47">
         <v>1</v>
       </c>
       <c r="H47" t="s">
-        <v>140</v>
+        <v>93</v>
       </c>
       <c r="I47" t="s">
-        <v>77</v>
+        <v>29</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="B48">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C48" t="s">
         <v>130</v>
       </c>
       <c r="D48" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="E48" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="F48" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="G48">
         <v>1</v>
       </c>
       <c r="H48" t="s">
-        <v>140</v>
+        <v>93</v>
       </c>
       <c r="I48" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="49" spans="1:9">
       <c r="A49">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="B49">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C49" t="s">
         <v>130</v>
       </c>
       <c r="D49" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="E49" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="F49" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="G49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H49" t="s">
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="I49" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
     </row>
     <row r="50" spans="1:9">
       <c r="A50">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="B50">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C50" t="s">
         <v>130</v>
       </c>
       <c r="D50" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="E50" t="s">
-        <v>138</v>
+        <v>165</v>
       </c>
       <c r="F50" t="s">
-        <v>139</v>
+        <v>166</v>
       </c>
       <c r="G50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H50" t="s">
-        <v>140</v>
+        <v>93</v>
       </c>
       <c r="I50" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
     </row>
     <row r="51" spans="1:9">
       <c r="A51">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="B51">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C51" t="s">
         <v>130</v>
       </c>
       <c r="D51" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="E51" t="s">
-        <v>138</v>
+        <v>165</v>
       </c>
       <c r="F51" t="s">
-        <v>139</v>
+        <v>166</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H51" t="s">
-        <v>140</v>
+        <v>93</v>
       </c>
       <c r="I51" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
     </row>
     <row r="52" spans="1:9">
       <c r="A52">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="B52">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C52" t="s">
         <v>130</v>
       </c>
       <c r="D52" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
       <c r="E52" t="s">
-        <v>138</v>
+        <v>168</v>
       </c>
       <c r="F52" t="s">
-        <v>139</v>
-      </c>
-      <c r="G52">
-        <v>1</v>
+        <v>166</v>
+      </c>
+      <c r="G52" t="s">
+        <v>18</v>
       </c>
       <c r="H52" t="s">
-        <v>140</v>
+        <v>93</v>
       </c>
       <c r="I52" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
     </row>
     <row r="53" spans="1:9">
       <c r="A53">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="B53">
-        <v>2013013630</v>
+        <v>2013037005</v>
       </c>
       <c r="C53" t="s">
         <v>130</v>
       </c>
       <c r="D53" t="s">
-        <v>137</v>
+        <v>169</v>
       </c>
       <c r="E53" t="s">
-        <v>138</v>
+        <v>170</v>
       </c>
       <c r="F53" t="s">
-        <v>139</v>
+        <v>171</v>
       </c>
       <c r="G53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H53" t="s">
-        <v>140</v>
+        <v>172</v>
       </c>
       <c r="I53" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
     </row>
     <row r="54" spans="1:9">
       <c r="A54">
-        <v>110</v>
+        <v>77</v>
       </c>
       <c r="B54">
         <v>2013013630</v>
       </c>
       <c r="C54" t="s">
-        <v>130</v>
+        <v>173</v>
       </c>
       <c r="D54" t="s">
-        <v>137</v>
+        <v>174</v>
       </c>
       <c r="E54" t="s">
-        <v>138</v>
+        <v>175</v>
       </c>
       <c r="F54" t="s">
-        <v>139</v>
+        <v>176</v>
       </c>
       <c r="G54">
         <v>1</v>
       </c>
       <c r="H54" t="s">
-        <v>140</v>
+        <v>85</v>
       </c>
       <c r="I54" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
     </row>
     <row r="55" spans="1:9">
       <c r="A55">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B55">
         <v>2013013630</v>
       </c>
       <c r="C55" t="s">
-        <v>130</v>
+        <v>173</v>
       </c>
       <c r="D55" t="s">
-        <v>137</v>
+        <v>177</v>
       </c>
       <c r="E55" t="s">
-        <v>138</v>
+        <v>178</v>
       </c>
       <c r="F55" t="s">
-        <v>139</v>
+        <v>179</v>
       </c>
       <c r="G55">
         <v>1</v>
       </c>
       <c r="H55" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
       <c r="I55" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56" spans="1:9">
       <c r="A56">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="B56">
-        <v>2013013630</v>
+        <v>2015132844</v>
       </c>
       <c r="C56" t="s">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="D56" t="s">
-        <v>137</v>
+        <v>181</v>
       </c>
       <c r="E56" t="s">
-        <v>138</v>
+        <v>182</v>
       </c>
       <c r="F56" t="s">
-        <v>139</v>
-      </c>
-      <c r="G56">
-        <v>1</v>
+        <v>183</v>
+      </c>
+      <c r="G56" t="s">
+        <v>18</v>
       </c>
       <c r="H56" t="s">
-        <v>140</v>
+        <v>184</v>
       </c>
       <c r="I56" t="s">
-        <v>77</v>
+        <v>19</v>
       </c>
     </row>
     <row r="57" spans="1:9">
       <c r="A57">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="B57">
-        <v>2013013630</v>
+        <v>2015132844</v>
       </c>
       <c r="C57" t="s">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="D57" t="s">
-        <v>137</v>
+        <v>185</v>
       </c>
       <c r="E57" t="s">
-        <v>138</v>
+        <v>186</v>
       </c>
       <c r="F57" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="G57">
         <v>1</v>
       </c>
       <c r="H57" t="s">
-        <v>140</v>
+        <v>188</v>
       </c>
       <c r="I57" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
     </row>
     <row r="58" spans="1:9">
       <c r="A58">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B58">
-        <v>2013013630</v>
+        <v>2015120792</v>
       </c>
       <c r="C58" t="s">
-        <v>130</v>
+        <v>189</v>
       </c>
       <c r="D58" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="E58" t="s">
-        <v>138</v>
+        <v>191</v>
       </c>
       <c r="F58" t="s">
-        <v>139</v>
-      </c>
-      <c r="G58">
-        <v>1</v>
+        <v>192</v>
+      </c>
+      <c r="G58" t="s">
+        <v>18</v>
       </c>
       <c r="H58" t="s">
-        <v>140</v>
+        <v>193</v>
       </c>
       <c r="I58" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9">
-      <c r="A59">
-        <v>115</v>
-      </c>
-      <c r="B59">
-        <v>2013013630</v>
-      </c>
-      <c r="C59" t="s">
-        <v>130</v>
-      </c>
-      <c r="D59" t="s">
-        <v>137</v>
-      </c>
-      <c r="E59" t="s">
-        <v>138</v>
-      </c>
-      <c r="F59" t="s">
-        <v>139</v>
-      </c>
-      <c r="G59">
-        <v>1</v>
-      </c>
-      <c r="H59" t="s">
-        <v>140</v>
-      </c>
-      <c r="I59" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9">
-      <c r="A60">
-        <v>116</v>
-      </c>
-      <c r="B60">
-        <v>2013013630</v>
-      </c>
-      <c r="C60" t="s">
-        <v>130</v>
-      </c>
-      <c r="D60" t="s">
-        <v>137</v>
-      </c>
-      <c r="E60" t="s">
-        <v>138</v>
-      </c>
-      <c r="F60" t="s">
-        <v>139</v>
-      </c>
-      <c r="G60">
-        <v>1</v>
-      </c>
-      <c r="H60" t="s">
-        <v>140</v>
-      </c>
-      <c r="I60" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9">
-      <c r="A61">
-        <v>117</v>
-      </c>
-      <c r="B61">
-        <v>2013013630</v>
-      </c>
-      <c r="C61" t="s">
-        <v>130</v>
-      </c>
-      <c r="D61" t="s">
-        <v>141</v>
-      </c>
-      <c r="E61" t="s">
-        <v>142</v>
-      </c>
-      <c r="F61" t="s">
-        <v>139</v>
-      </c>
-      <c r="G61">
-        <v>1</v>
-      </c>
-      <c r="H61" t="s">
-        <v>140</v>
-      </c>
-      <c r="I61" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9">
-      <c r="A62">
-        <v>82</v>
-      </c>
-      <c r="B62">
-        <v>2015132844</v>
-      </c>
-      <c r="C62" t="s">
-        <v>143</v>
-      </c>
-      <c r="D62" t="s">
-        <v>144</v>
-      </c>
-      <c r="E62" t="s">
-        <v>145</v>
-      </c>
-      <c r="F62" t="s">
-        <v>146</v>
-      </c>
-      <c r="G62" t="s">
-        <v>18</v>
-      </c>
-      <c r="H62" t="s">
-        <v>147</v>
-      </c>
-      <c r="I62" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9">
-      <c r="A63">
-        <v>83</v>
-      </c>
-      <c r="B63">
-        <v>2015132844</v>
-      </c>
-      <c r="C63" t="s">
-        <v>143</v>
-      </c>
-      <c r="D63" t="s">
-        <v>148</v>
-      </c>
-      <c r="E63" t="s">
-        <v>149</v>
-      </c>
-      <c r="F63" t="s">
-        <v>150</v>
-      </c>
-      <c r="G63">
-        <v>1</v>
-      </c>
-      <c r="H63" t="s">
-        <v>151</v>
-      </c>
-      <c r="I63" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>